<commit_message>
Add restaurant data: 24 restaurants scraped from Queretaro via Apify
</commit_message>
<xml_diff>
--- a/sheets/restaurants.xlsx
+++ b/sheets/restaurants.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,6 +503,1484 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ChIJpcZ3ngBF04URV43PimP-zQE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>130 Grados Steakhouse Querétaro</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Brasil 29, Lomas de Queretaro, 76190 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+52 442 847 3813</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>http://www.130grados.mx/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>20.5721201</v>
+      </c>
+      <c r="P2" t="n">
+        <v>-100.4059284</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=130%20Grados%20Steakhouse%20Quer%C3%A9taro&amp;query_place_id=ChIJpcZ3ngBF04URV43PimP-zQE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ChIJCzisuB5b04URvDmfy2FBl2E</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hacienda Laborcilla</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Prol. Corregidora Nte. 911 bis, Quinta la Laborcilla, 76168 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+52 442 245 2439</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>http://www.haciendalaborcilla.com/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10731</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>20.6129347</v>
+      </c>
+      <c r="P3" t="n">
+        <v>-100.388559</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hacienda%20Laborcilla&amp;query_place_id=ChIJCzisuB5b04URvDmfy2FBl2E</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ChIJb80rszdb04UR0pVuHwUYO0c</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cabo Sierra</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Prol. Bernardo Quintana 30, Calesa, 76020 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+52 442 488 8043</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>http://www.cabosierra.com/?utm_source=google&amp;utm_medium=wix_google_business_profile&amp;utm_campaign=16537793470922407642</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>513</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>20.5994931</v>
+      </c>
+      <c r="P4" t="n">
+        <v>-100.3747695</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Cabo%20Sierra&amp;query_place_id=ChIJb80rszdb04UR0pVuHwUYO0c</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ChIJ3chRrS1b04URaexj2wsDFmw</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Carranza 50</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>C. Venustiano Carranza 50, La Santa Cruz, Centro, 76020 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+52 442 212 3031</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>http://www.carranza50.com.mx/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2392</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>20.5930346</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-100.3862707</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Carranza%2050&amp;query_place_id=ChIJ3chRrS1b04URaexj2wsDFmw</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ChIJsdKPgvpE04URyva84BL22Gw</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Chucho El Roto</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Av. Luis Pasteur Sur 16, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>+52 442 212 4295</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://www.chuchoelroto.com.mx/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10107</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>20.5927545</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-100.3893559</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Chucho%20El%20Roto&amp;query_place_id=ChIJsdKPgvpE04URyva84BL22Gw</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ChIJAaW17Cpb04UROK2iVI57Gmw</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tikua - SouthEast Mexican cuisine</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>C. Ignacio Allende Sur 13, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>+52 442 403 4677</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>http://www.tikua.mx/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4225</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>20.5910131</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-100.3932327</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Tikua%20-%20SouthEast%20Mexican%20cuisine&amp;query_place_id=ChIJAaW17Cpb04UROK2iVI57Gmw</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ChIJZ3b7Bjdb04URPYwOrZTi3Lc</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>il Duomo Cocina Italiana</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Blvd. Bernardo Quintana Arrioja 32, Calesa, 76020 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>+52 442 213 7768</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>http://www.grupopasta.com/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2689</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>20.5997029</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-100.3748168</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=il%20Duomo%20Cocina%20Italiana&amp;query_place_id=ChIJZ3b7Bjdb04URPYwOrZTi3Lc</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ChIJE-AvmylF04URNwcyzF9qYQI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Argentilia Querétaro</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>59, Av. Constituyentes, Casa Blanca, 76030 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>+52 442 215 1005</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://argentilia.mx/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3336</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>20.5820892</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-100.3970316</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Argentilia%20Quer%C3%A9taro&amp;query_place_id=ChIJE-AvmylF04URNwcyzF9qYQI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ChIJVVWR5klb04UR2fJ5ydGVLrM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ziracco</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Calz. de los Arcos 161, Calesa, 76020 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+52 442 538 2371</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://ziracco.com/</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>775</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>20.5973504</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-100.3717871</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Ziracco&amp;query_place_id=ChIJVVWR5klb04UR2fJ5ydGVLrM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ChIJO1uX_Ttb04UR7TTOzAfXEiQ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mochomos Querétaro</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Prol. Bernardo Quintana 5260-1D, Colinas del Parque, 76140 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>+52 442 902 6179</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://mochomos.mx/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2453</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>20.6070957</v>
+      </c>
+      <c r="P11" t="n">
+        <v>-100.3777482</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Mochomos%20Quer%C3%A9taro&amp;query_place_id=ChIJO1uX_Ttb04UR7TTOzAfXEiQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ChIJEXP8_ypb04URcpMHadwogVE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Restaurante Bar Hank's Querétaro</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Acceso por la, Calle Benito Juárez Sur, Pl. Constitución 7, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>+52 442 214 2620</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.hanksmexico.com/</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3958</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="b">
+        <v>0</v>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>20.5919303</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-100.3918839</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Restaurante%20Bar%20Hank's%20Quer%C3%A9taro&amp;query_place_id=ChIJEXP8_ypb04URcpMHadwogVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ChIJhWjd3v5b04URI2EQ_O9n4Jo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>La Unica Querétaro</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Calz. de los Arcos 33, Bosques del Acueducto, 76020 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>+52 442 213 5883</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>http://www.launica.mx/</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>745</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="b">
+        <v>0</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>20.5941509</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-100.3763299</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=La%20Unica%20Quer%C3%A9taro&amp;query_place_id=ChIJhWjd3v5b04URI2EQ_O9n4Jo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ChIJDykoE8U_04URB3gu4vtHwO4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Restaurante Fogón Zapoteco en Centro Querétaro</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>C. Francisco I. Madero Poniente 86, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>+52 442 464 7128</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/fogonzapoteco/</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1360</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="b">
+        <v>0</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20.5907267</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-100.397523</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Restaurante%20Fog%C3%B3n%20Zapoteco%20en%20Centro%20Quer%C3%A9taro&amp;query_place_id=ChIJDykoE8U_04URB3gu4vtHwO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ChIJNSVTJgFa04URGuB0DewnHwg</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Santo Mar</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>San Luis Potosí - Santiago de Querétaro, 76127 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>+52 442 747 3131</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://santomar.shop/</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2884</v>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>20.6748431</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-100.4378469</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Santo%20Mar&amp;query_place_id=ChIJNSVTJgFa04URGuB0DewnHwg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ChIJhysq59Za04URYQZLIP37JHo</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Oliva</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>76000, Av. Universidad 37 a, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>+52 442 212 7059</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/OLIVA-restaurante-1463838460302252/?fref=ts</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>819</v>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>20.5971743</v>
+      </c>
+      <c r="P16" t="n">
+        <v>-100.3986409</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Oliva&amp;query_place_id=ChIJhysq59Za04URYQZLIP37JHo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ChIJs3TKailF04URS7ubzvmMgz4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Parrilla Leonesa</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Av. Constituyentes Ote. 138, Panamericano, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>+52 442 216 2123</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>http://www.parrillaleonesa.com.mx/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5253</v>
+      </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>20.5811348</v>
+      </c>
+      <c r="P17" t="n">
+        <v>-100.3992154</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Parrilla%20Leonesa&amp;query_place_id=ChIJs3TKailF04URS7ubzvmMgz4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ChIJW2KAkBBa04URjVJYsh2yuz4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Hacienda El Salitre</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rafael Osuna SN, Raquet Club, 76127 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>+52 442 825 8866</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.elsalitre.mx/</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3118</v>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" t="b">
+        <v>0</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>20.6669695</v>
+      </c>
+      <c r="P18" t="n">
+        <v>-100.4266499</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hacienda%20El%20Salitre&amp;query_place_id=ChIJW2KAkBBa04URjVJYsh2yuz4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ChIJpxfxVTlb04URT-v_El5BX-M</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>La Bocha</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Prol. Bernardo Quintana 5260, Residencial Viveros, 76140 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>+52 442 245 3142</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/labochaqro</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2067</v>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="b">
+        <v>0</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>20.6072932</v>
+      </c>
+      <c r="P19" t="n">
+        <v>-100.3777635</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=La%20Bocha&amp;query_place_id=ChIJpxfxVTlb04URT-v_El5BX-M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ChIJAQeR59VE04URIdDTJTt_uVI</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tacos El Pata</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fray Pedro de Gante 8, Cimatario, 76030 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>+52 442 224 1376</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>http://tacoselpata.com/</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10285</v>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="b">
+        <v>0</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>20.5838375</v>
+      </c>
+      <c r="P20" t="n">
+        <v>-100.3935783</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Tacos%20El%20Pata&amp;query_place_id=ChIJAQeR59VE04URIdDTJTt_uVI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ChIJG7laIpha04UR0lN4WWAFl4g</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Restaurante 1810</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>And. Libertad 62, Centro, 76000 Santiago de Querétaro, Qro., Mexico</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>+52 442 214 3324</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://restaurante1810.wordpress.com/nuestro-menu/</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2926</v>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="b">
+        <v>0</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>20.5926335</v>
+      </c>
+      <c r="P21" t="n">
+        <v>-100.3894769</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Restaurante%201810&amp;query_place_id=ChIJG7laIpha04UR0lN4WWAFl4g</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ChIJvRp3sT5-j4AR6-HtouO7E_s</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>El Rey Taquiza Artesanal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2491 Mission St, San Francisco, CA 94110</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(415) 796-2139</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.elreytaquiza.com/</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>265</v>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>37.7572679</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-122.418732</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=El%20Rey%20Taquiza%20Artesanal&amp;query_place_id=ChIJvRp3sT5-j4AR6-HtouO7E_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ChIJb8aQHACBhYAR4IOvll5mgzk</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Al Pastor Papi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>232 O'Farrell St, San Francisco, CA 94102</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>124</v>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>37.7864848</v>
+      </c>
+      <c r="P23" t="n">
+        <v>-122.4086079</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Al%20Pastor%20Papi&amp;query_place_id=ChIJb8aQHACBhYAR4IOvll5mgzk</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ChIJHy305b4zjoARobO-3mW0K-8</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>mariscos la ceiba monterrey rd</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4100 Monterey Rd #108, San Jose, CA 95111</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>(669) 350-4612</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>http://mariscoslaceiba.com/</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G24" t="n">
+        <v>75</v>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" t="b">
+        <v>0</v>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>37.2793053</v>
+      </c>
+      <c r="P24" t="n">
+        <v>-121.8347287</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=mariscos%20la%20ceiba%20monterrey%20rd&amp;query_place_id=ChIJHy305b4zjoARobO-3mW0K-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ChIJqXXgleHDyIAR5re4RR2tRWw</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>El Borrego Dorado</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2605 S Eastern Ave, Las Vegas, NV 89169</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(702) 624-2339</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>http://elborregodorado.weebly.com/</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>28</v>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>36.1419503</v>
+      </c>
+      <c r="P25" t="n">
+        <v>-115.1200566</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=El%20Borrego%20Dorado&amp;query_place_id=ChIJqXXgleHDyIAR5re4RR2tRWw</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>